<commit_message>
Update attendees for quiz: new — fevin@gmail.com
</commit_message>
<xml_diff>
--- a/quizzes/new/attendees.xlsx
+++ b/quizzes/new/attendees.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M1"/>
+  <dimension ref="A1:M2"/>
   <cols>
     <col min="1" max="1" width="30.83203125" customWidth="1"/>
     <col min="2" max="2" width="20.83203125" customWidth="1"/>
@@ -455,9 +455,50 @@
         <v>Grade</v>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>fevin@gmail.com</v>
+      </c>
+      <c r="B2" t="str">
+        <v>as</v>
+      </c>
+      <c r="C2" t="str">
+        <v>new</v>
+      </c>
+      <c r="D2" t="str">
+        <v>8/13/2026, 12:12:47 AM</v>
+      </c>
+      <c r="E2">
+        <v>2</v>
+      </c>
+      <c r="F2">
+        <v>1</v>
+      </c>
+      <c r="G2">
+        <v>0</v>
+      </c>
+      <c r="H2">
+        <v>1</v>
+      </c>
+      <c r="I2">
+        <v>1</v>
+      </c>
+      <c r="J2">
+        <v>2</v>
+      </c>
+      <c r="K2">
+        <v>0</v>
+      </c>
+      <c r="L2" t="str">
+        <v>0.00</v>
+      </c>
+      <c r="M2" t="str">
+        <v>F</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M2"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>